<commit_message>
added new test files at 9:41 PM on 6-May-2026
</commit_message>
<xml_diff>
--- a/testdata/login_data.xlsx
+++ b/testdata/login_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srout\Desktop\SONALI\Personal\SelfLearning\PythonWithSeleniumTraining\udemy\ZSeleniumFramework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13C42F8D-B642-43D3-9633-659F01AA0547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FBF6A75-33BA-46FA-9BA2-3980B3B8F437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="580" windowWidth="11290" windowHeight="8220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>username</t>
   </si>
@@ -40,9 +40,6 @@
   </si>
   <si>
     <t>admin123</t>
-  </si>
-  <si>
-    <t>AAAAA</t>
   </si>
 </sst>
 </file>
@@ -405,13 +402,13 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>5</v>
+      <c r="A3">
+        <v>11111</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="2" t="b">
+      <c r="C3" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated test files at 10:56 PM 6-May-2026
</commit_message>
<xml_diff>
--- a/testdata/login_data.xlsx
+++ b/testdata/login_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\srout\Desktop\SONALI\Personal\SelfLearning\PythonWithSeleniumTraining\udemy\ZSeleniumFramework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FBF6A75-33BA-46FA-9BA2-3980B3B8F437}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CC42F6-F1F0-425C-A2D9-AA15F5724E2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>username</t>
   </si>
@@ -371,7 +371,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.1796875" bestFit="1" customWidth="1"/>
@@ -401,17 +401,6 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>11111</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="b">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>